<commit_message>
fix import excel for product, accountant and fix create product request history
</commit_message>
<xml_diff>
--- a/frontend/huongvantra-web-client/public/templates/phieu-nhap-kho-excel-tt200.xlsx
+++ b/frontend/huongvantra-web-client/public/templates/phieu-nhap-kho-excel-tt200.xlsx
@@ -202,31 +202,30 @@
     <font>
       <color theme="1"/>
       <family val="2"/>
-      <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
     </font>
     <font>
       <i/>
-      <sz val="11"/>
+      <sz val="12"/>
       <name val="Times New Roman"/>
     </font>
     <font>
       <b/>
       <color rgb="FF356647"/>
-      <sz val="11"/>
+      <sz val="12"/>
       <name val="Times New Roman"/>
     </font>
     <font>
       <i/>
       <color rgb="FF666666"/>
-      <sz val="9"/>
+      <sz val="12"/>
       <name val="Times New Roman"/>
     </font>
     <font>
       <b/>
       <color rgb="FF356647"/>
-      <sz val="20"/>
+      <sz val="12.5"/>
       <name val="Times New Roman"/>
     </font>
     <font>
@@ -234,7 +233,7 @@
       <name val="Times New Roman"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <name val="Times New Roman"/>
     </font>
     <font>
@@ -245,35 +244,35 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
+      <sz val="12"/>
       <name val="Times New Roman"/>
     </font>
     <font>
       <i/>
       <color rgb="FF888888"/>
-      <sz val="9"/>
+      <sz val="12"/>
       <name val="Times New Roman"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="12"/>
       <name val="Times New Roman"/>
     </font>
     <font>
       <i/>
       <color rgb="FF777777"/>
-      <sz val="9"/>
+      <sz val="12"/>
       <name val="Times New Roman"/>
     </font>
     <font>
       <b/>
       <color rgb="FF356647"/>
-      <sz val="14"/>
-      <name val="Calibri"/>
+      <sz val="12.5"/>
+      <name val="Times New Roman"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
     </font>
   </fonts>
   <fills count="15">

</xml_diff>